<commit_message>
LLM call failed: ResponseError: {"error":{"code":400,"message":"request (34344 tokens) exceeds the available context size (32768 tokens), try increasing it","type":"exceed_context_size_error","n_prompt_tokens":34344,"n_ctx":32768}} (status code: 400)
</commit_message>
<xml_diff>
--- a/라만_벤치마크.xlsx
+++ b/라만_벤치마크.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\gemma_raman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB2984D8-B3FA-457A-8B69-042797635F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9ADA25A4-AA81-4D0D-B3A7-EE006D6CD2EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="8085" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Task_채점기준" sheetId="1" r:id="rId1"/>

</xml_diff>